<commit_message>
deleted:    .~lock.player_sm.xlsx# deleted:    .~lock.team_sm.xlsx# modified:   freshness.xlsx modified:   goDTL.xlsx deleted:    player_sm.xlsx new file:   playersm.xlsx deleted:    team_sm.xlsx new file:   teamsm.xlsx
</commit_message>
<xml_diff>
--- a/freshness.xlsx
+++ b/freshness.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steve\Downloads\1-3-26-Game Report\1-3-26 game report for Liam\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steve\Downloads\1-10-26-Sabres Game Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51198A39-D8FC-4964-9693-A99162EC2B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AC0B996-5CAD-4C18-9C0F-561D086127A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,58 +43,58 @@
     <t>Ukko-Pekka Luukkonen</t>
   </si>
   <si>
+    <t>Tage Thompson</t>
+  </si>
+  <si>
+    <t>Mattias Samuelsson</t>
+  </si>
+  <si>
+    <t>Jason Zucker</t>
+  </si>
+  <si>
+    <t>Bowen Byram</t>
+  </si>
+  <si>
+    <t>Owen Power</t>
+  </si>
+  <si>
+    <t>Josh Norris</t>
+  </si>
+  <si>
+    <t>Rasmus Dahlin</t>
+  </si>
+  <si>
+    <t>Peyton Krebs</t>
+  </si>
+  <si>
+    <t>Zach Metsa</t>
+  </si>
+  <si>
+    <t>Beck Malenstyn</t>
+  </si>
+  <si>
     <t>Josh Doan</t>
   </si>
   <si>
-    <t>Rasmus Dahlin</t>
-  </si>
-  <si>
-    <t>Josh Norris</t>
+    <t>Jordan Greenway</t>
+  </si>
+  <si>
+    <t>Alex Tuch</t>
+  </si>
+  <si>
+    <t>Ryan McLeod</t>
+  </si>
+  <si>
+    <t>Noah Ostlund</t>
+  </si>
+  <si>
+    <t>Jacob Bryson</t>
+  </si>
+  <si>
+    <t>Jack Quinn</t>
   </si>
   <si>
     <t>Zach Benson</t>
-  </si>
-  <si>
-    <t>Tage Thompson</t>
-  </si>
-  <si>
-    <t>Mattias Samuelsson</t>
-  </si>
-  <si>
-    <t>Alex Tuch</t>
-  </si>
-  <si>
-    <t>Peyton Krebs</t>
-  </si>
-  <si>
-    <t>Ryan McLeod</t>
-  </si>
-  <si>
-    <t>Jacob Bryson</t>
-  </si>
-  <si>
-    <t>Bowen Byram</t>
-  </si>
-  <si>
-    <t>Zach Metsa</t>
-  </si>
-  <si>
-    <t>Owen Power</t>
-  </si>
-  <si>
-    <t>Jack Quinn</t>
-  </si>
-  <si>
-    <t>Noah Ostlund</t>
-  </si>
-  <si>
-    <t>Jordan Greenway</t>
-  </si>
-  <si>
-    <t>Josh Dunne</t>
-  </si>
-  <si>
-    <t>Beck Malenstyn</t>
   </si>
 </sst>
 </file>
@@ -449,7 +449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{535CA78B-7A84-4E37-A947-D00FE98D5581}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFAF21F3-47FD-42B1-AE99-15CA746044FA}">
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
@@ -481,22 +481,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>46025</v>
+        <v>46032</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="2">
-        <v>190.42</v>
+        <v>270.28399999999999</v>
       </c>
       <c r="D2" s="2">
-        <v>86.712500000000006</v>
+        <v>91.086200000000005</v>
       </c>
       <c r="E2" s="2">
-        <v>-11.950200000000001</v>
+        <v>-23.563800000000001</v>
       </c>
       <c r="F2" s="2">
-        <v>-32.4131</v>
+        <v>-47.479199999999999</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -504,16 +504,16 @@
         <v>7</v>
       </c>
       <c r="C3" s="2">
-        <v>182.01900000000001</v>
+        <v>237.9717</v>
       </c>
       <c r="D3" s="2">
-        <v>95.469200000000001</v>
+        <v>101.4499</v>
       </c>
       <c r="E3" s="2">
-        <v>-11.898099999999999</v>
+        <v>-13.738200000000001</v>
       </c>
       <c r="F3" s="2">
-        <v>-23.591000000000001</v>
+        <v>-35.954999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -521,16 +521,16 @@
         <v>8</v>
       </c>
       <c r="C4" s="2">
-        <v>178.64410000000001</v>
+        <v>234.53129999999999</v>
       </c>
       <c r="D4" s="2">
-        <v>94.531999999999996</v>
+        <v>96.796300000000002</v>
       </c>
       <c r="E4" s="2">
-        <v>-10.477499999999999</v>
+        <v>-16.0609</v>
       </c>
       <c r="F4" s="2">
-        <v>-32.219799999999999</v>
+        <v>-36.960700000000003</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -538,16 +538,16 @@
         <v>9</v>
       </c>
       <c r="C5" s="2">
-        <v>170.9427</v>
+        <v>234.4624</v>
       </c>
       <c r="D5" s="2">
-        <v>78.517700000000005</v>
+        <v>64.359099999999998</v>
       </c>
       <c r="E5" s="2">
-        <v>-18.683399999999999</v>
+        <v>-34.685400000000001</v>
       </c>
       <c r="F5" s="2">
-        <v>-27.684799999999999</v>
+        <v>-68.394400000000005</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -555,16 +555,16 @@
         <v>10</v>
       </c>
       <c r="C6" s="2">
-        <v>170.89840000000001</v>
+        <v>230.1866</v>
       </c>
       <c r="D6" s="2">
-        <v>89.590999999999994</v>
+        <v>99.497699999999995</v>
       </c>
       <c r="E6" s="2">
-        <v>-14.5913</v>
+        <v>-15.034599999999999</v>
       </c>
       <c r="F6" s="2">
-        <v>-23.822099999999999</v>
+        <v>-34.86</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -572,16 +572,16 @@
         <v>11</v>
       </c>
       <c r="C7" s="2">
-        <v>169.09549999999999</v>
+        <v>226.97829999999999</v>
       </c>
       <c r="D7" s="2">
-        <v>99.004499999999993</v>
+        <v>104.1611</v>
       </c>
       <c r="E7" s="2">
-        <v>0.50129999999999997</v>
+        <v>-13.3919</v>
       </c>
       <c r="F7" s="2">
-        <v>-8.2242999999999995</v>
+        <v>-31.619199999999999</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -589,16 +589,16 @@
         <v>12</v>
       </c>
       <c r="C8" s="2">
-        <v>164.49</v>
+        <v>224.57910000000001</v>
       </c>
       <c r="D8" s="2">
-        <v>94.394300000000001</v>
+        <v>84.384799999999998</v>
       </c>
       <c r="E8" s="2">
-        <v>-6.2405999999999997</v>
+        <v>-29.1951</v>
       </c>
       <c r="F8" s="2">
-        <v>-11.8713</v>
+        <v>-47.091999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -606,16 +606,16 @@
         <v>13</v>
       </c>
       <c r="C9" s="2">
-        <v>163.1335</v>
+        <v>223.2286</v>
       </c>
       <c r="D9" s="2">
-        <v>91.227500000000006</v>
+        <v>96.482299999999995</v>
       </c>
       <c r="E9" s="2">
-        <v>-4.2239000000000004</v>
+        <v>-15.7256</v>
       </c>
       <c r="F9" s="2">
-        <v>-13.192299999999999</v>
+        <v>-34.292099999999998</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -623,16 +623,16 @@
         <v>14</v>
       </c>
       <c r="C10" s="2">
-        <v>162.28389999999999</v>
+        <v>207.88669999999999</v>
       </c>
       <c r="D10" s="2">
-        <v>88.631699999999995</v>
+        <v>91.334400000000002</v>
       </c>
       <c r="E10" s="2">
-        <v>-2.9403000000000001</v>
+        <v>-14.7995</v>
       </c>
       <c r="F10" s="2">
-        <v>-11.9107</v>
+        <v>-33.312199999999997</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -640,16 +640,16 @@
         <v>15</v>
       </c>
       <c r="C11" s="2">
-        <v>161.1147</v>
+        <v>205.97669999999999</v>
       </c>
       <c r="D11" s="2">
-        <v>96.989599999999996</v>
+        <v>86.329899999999995</v>
       </c>
       <c r="E11" s="2">
-        <v>-1.8033999999999999</v>
+        <v>-25.095600000000001</v>
       </c>
       <c r="F11" s="2">
-        <v>-7.5792999999999999</v>
+        <v>-40.354900000000001</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -657,16 +657,16 @@
         <v>16</v>
       </c>
       <c r="C12" s="2">
-        <v>158.31710000000001</v>
+        <v>203.44120000000001</v>
       </c>
       <c r="D12" s="2">
-        <v>72.296599999999998</v>
+        <v>97.272599999999997</v>
       </c>
       <c r="E12" s="2">
-        <v>-4.6923000000000004</v>
+        <v>-16.196300000000001</v>
       </c>
       <c r="F12" s="2">
-        <v>-18.9818</v>
+        <v>-31.918199999999999</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -674,16 +674,16 @@
         <v>17</v>
       </c>
       <c r="C13" s="2">
-        <v>155.08949999999999</v>
+        <v>201.64160000000001</v>
       </c>
       <c r="D13" s="2">
-        <v>96.491500000000002</v>
+        <v>97.900199999999998</v>
       </c>
       <c r="E13" s="2">
-        <v>-1.3018000000000001</v>
+        <v>-14.5197</v>
       </c>
       <c r="F13" s="2">
-        <v>-7.8194999999999997</v>
+        <v>-24.975200000000001</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -691,16 +691,16 @@
         <v>18</v>
       </c>
       <c r="C14" s="2">
-        <v>147.51689999999999</v>
+        <v>201.00960000000001</v>
       </c>
       <c r="D14" s="2">
-        <v>81.752799999999993</v>
+        <v>79.442400000000006</v>
       </c>
       <c r="E14" s="2">
-        <v>-17.7453</v>
+        <v>-29.466899999999999</v>
       </c>
       <c r="F14" s="2">
-        <v>-21.684100000000001</v>
+        <v>-49.169400000000003</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -708,16 +708,16 @@
         <v>19</v>
       </c>
       <c r="C15" s="2">
-        <v>147.1174</v>
+        <v>200.7551</v>
       </c>
       <c r="D15" s="2">
-        <v>102.4358</v>
+        <v>93.316699999999997</v>
       </c>
       <c r="E15" s="2">
-        <v>-5.4341999999999997</v>
+        <v>-13.2682</v>
       </c>
       <c r="F15" s="2">
-        <v>-9.1809999999999992</v>
+        <v>-30.045500000000001</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -725,16 +725,16 @@
         <v>20</v>
       </c>
       <c r="C16" s="2">
-        <v>146.03120000000001</v>
+        <v>200.05119999999999</v>
       </c>
       <c r="D16" s="2">
-        <v>104.8629</v>
+        <v>97.546199999999999</v>
       </c>
       <c r="E16" s="2">
-        <v>-5.9893999999999998</v>
+        <v>-7.2577999999999996</v>
       </c>
       <c r="F16" s="2">
-        <v>-8.6918000000000006</v>
+        <v>-21.9404</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
@@ -742,16 +742,16 @@
         <v>21</v>
       </c>
       <c r="C17" s="2">
-        <v>141.6688</v>
+        <v>199.67920000000001</v>
       </c>
       <c r="D17" s="2">
-        <v>82.133099999999999</v>
+        <v>86.736800000000002</v>
       </c>
       <c r="E17" s="2">
-        <v>-14.6348</v>
+        <v>-24.550799999999999</v>
       </c>
       <c r="F17" s="2">
-        <v>-18.62</v>
+        <v>-41.089100000000002</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -759,16 +759,16 @@
         <v>22</v>
       </c>
       <c r="C18" s="2">
-        <v>122.90389999999999</v>
+        <v>190.125</v>
       </c>
       <c r="D18" s="2">
-        <v>72.663300000000007</v>
+        <v>76.251000000000005</v>
       </c>
       <c r="E18" s="2">
-        <v>-10.8248</v>
+        <v>-18.353000000000002</v>
       </c>
       <c r="F18" s="2">
-        <v>-20.567599999999999</v>
+        <v>-36.383400000000002</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
@@ -776,16 +776,16 @@
         <v>23</v>
       </c>
       <c r="C19" s="2">
-        <v>122.693</v>
+        <v>183.57640000000001</v>
       </c>
       <c r="D19" s="2">
-        <v>78.096400000000003</v>
+        <v>105.97239999999999</v>
       </c>
       <c r="E19" s="2">
-        <v>-13.649800000000001</v>
+        <v>-7.8278999999999996</v>
       </c>
       <c r="F19" s="2">
-        <v>-16.901900000000001</v>
+        <v>-14.8095</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
@@ -793,16 +793,16 @@
         <v>24</v>
       </c>
       <c r="C20" s="2">
-        <v>109.9937</v>
+        <v>134.923</v>
       </c>
       <c r="D20" s="2">
-        <v>93.763300000000001</v>
+        <v>91.335599999999999</v>
       </c>
       <c r="E20" s="2">
-        <v>-2.7917000000000001</v>
+        <v>-12.3734</v>
       </c>
       <c r="F20" s="2">
-        <v>6.3299999999999995E-2</v>
+        <v>-14.1212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>